<commit_message>
Atualização diária das Tabelas.
Atualizando Tabelas do sistema data 17/12/2025.
Atualização do arquivo __init__.cpython-313.ptc
</commit_message>
<xml_diff>
--- a/Arquivos/balanco.xlsx
+++ b/Arquivos/balanco.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="2" min="1" max="1"/>
@@ -1897,6 +1897,38 @@
         <v>-10.45</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>17/12/2025</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>860</v>
+      </c>
+      <c r="C92" t="n">
+        <v>308.35</v>
+      </c>
+      <c r="D92" t="n">
+        <v>551.65</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>17/12/2025</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>227.33</v>
+      </c>
+      <c r="D93" t="n">
+        <v>-227.33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização das Tabelas e adição de bat para chamada no terminal do prompt de comando.
</commit_message>
<xml_diff>
--- a/Arquivos/balanco.xlsx
+++ b/Arquivos/balanco.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="2" min="1" max="1"/>
@@ -1929,6 +1929,86 @@
         <v>-227.33</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>18/12/2025</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" t="n">
+        <v>146</v>
+      </c>
+      <c r="D94" t="n">
+        <v>-146</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>19/12/2025</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>120</v>
+      </c>
+      <c r="D95" t="n">
+        <v>-120</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>19/12/2025</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="D96" t="n">
+        <v>-16.06</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20/12/2025</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D97" t="n">
+        <v>-4.5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>21/12/2025</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="n">
+        <v>30.07</v>
+      </c>
+      <c r="D98" t="n">
+        <v>-30.07</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>

</xml_diff>